<commit_message>
Use uploaded Etagi templates from input/ and fill underscore fields
- Find templates in equipment-templates/input/ (user upload location)
- Fill Модель/Серийный/Инвентарный/Локация blanks from AI xlsx data
- Preserve full template text for personnel use

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/TEST_Sample_Device_Package.xlsx
+++ b/equipment-templates/output/TEST_Sample_Device_Package.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -431,156 +431,685 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ИНВЕНТАРНАЯ КАРТОЧКА ОРГТЕХНИКИ</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Организация: Этажи</t>
+          <t xml:space="preserve">КАРТОЧКА АППАРАТА № 67+    Дата: 22.06.2026  </t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr"/>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Инженеры: Антон / Александр</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Дата составления: 22.06.2026</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>№ п/п: 1</t>
-        </is>
-      </c>
+      <c r="A5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr"/>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>1. ИДЕНТИФИКАЦИЯ</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Инвентарный номер: 67+</t>
+          <t>───────────────────────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Марка / модель: Kyocera ECOSYS M3040dn</t>
+          <t xml:space="preserve">Модель:                  Kyocera ECOSYS M3040dn               </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Серийный номер: LS67Y43279</t>
+          <t xml:space="preserve">Серийный номер:          LS67Y43279                           </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Место размещения: Риелторы (Тюмень)</t>
+          <t xml:space="preserve">Инвентарный номер:       67+                                  </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Офис: Тюмень</t>
+          <t xml:space="preserve">Локация (офис/кабинет):  Риелторы (Тюмень)                    </t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>Подразделение: Риелторы</t>
-        </is>
-      </c>
+      <c r="A12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr"/>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>2. РЕКВИЗИТЫ ДЛЯ АНАЛИЗА</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Счетчик (предыдущий месяц): 272339</t>
+          <t>───────────────────────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Счетчик (отчетный месяц): 272864</t>
+          <t>IP-адрес:                _____________________________________</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Кол-во отпечатков: 525</t>
+          <t>MAC-адрес:               _____________________________________</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Модель картриджа:        _____________________________________</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ответственный сотрудник: </t>
+          <t>Текущий ресурс картриджа (%): ________________________________</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr"/>
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Версия прошивки:         _____________________________________</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Состояние оборудования: Исправно / Неисправно</t>
+          <t>Дата последнего ТО:      _____________________________________</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Примечание:</t>
+          <t>Дата последней замены ЗИП: ___________________________________</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr"/>
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Ответственный у Заказчика: ___________________________________</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>Материально ответственное лицо: __________________ / __________________</t>
+          <t>Контакт (тел/email):     _____________________________________</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>Инвентаризатор: __________________ / __________________</t>
-        </is>
-      </c>
+      <c r="A24" s="1" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Подписи. М.П.</t>
+          <t>3. СЧЕТЧИКИ</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="inlineStr"/>
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Общий пробег (Total):    272864       стр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>Ч/Б:                     ____________ стр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Цветной:                 ____________ стр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Сканер:                  ____________ стр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Пробег с последнего ТО:  525          стр.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>4. ФИЗИЧЕСКОЕ СОСТОЯНИЕ (отметить ✓ или ✗)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Корпус без трещин, крышки закрываются</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Лоток подачи бумаги: ролики чистые, не лысые, пружины целые</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Лоток выхода: флажки/направляющие целые</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Дуплекс-модуль: нет замятий, засохшего тонера</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Внутренность: нет рассыпанного тонера, бумаги, скрепок</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Кабель питания / USB — целые, с запасом</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Шум при работе: нет треска, скрежета, вибрации</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>5. КАЧЕСТВО ПЕЧАТИ (распечатать тестовую страницу из меню)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Равномерная плотность по всей странице</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Нет вертикальных полос / точек / фона</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Нет "волн" и повторяющихся дефектов (шаг дефекта: _____ мм)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Регистрация листа ровная (текст не уходит вбок)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Тонер закреплен (не смазывается пальцем)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>6. КАЧЕСТВО СКАНИРОВАНИЯ (протестировать на A4 и A3 если есть ADF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>[ ] ADF захватывает лист без перекоса</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>[ ] На скане нет полос (проверить стекло и зеркало)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Скан в сетевую папку / на email работает</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Двустороннее сканирование работает (если есть)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>7. СУБЪЕКТИВНАЯ ОЦЕНКА СОСТОЯНИЯ (1-5 баллов)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>Шкала оценки:</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1 — Критическое (не работает / требует срочного ремонта)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2 — Плохое (работает с перебоями / явные дефекты качества)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3 — Удовлетворительное (работает, но требует внимания/ТО)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4 — Хорошее (работает стабильно, мелкие замечания)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5 — Отличное (идеальное состояние, как новый)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t>Физическое состояние:    [ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t>Качество печати:         [ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>Качество сканирования:   [ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t>Общая оценка:            [ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t>Комментарий к оценке:</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t>________________________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t>________________________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr">
+        <is>
+          <t>8. ЗАМЕЧЕНИЯ И "БОЛЯЧКИ" (свободное описание)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>________________________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>________________________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr">
+        <is>
+          <t>________________________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr">
+        <is>
+          <t>9. ПЛАН ДЕЙСТВИЙ (отметить все применимые пункты)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr">
+        <is>
+          <t>───────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr">
+        <is>
+          <t>[ 1 ] Не требует действий — аппарат в рабочем состоянии</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="inlineStr">
+        <is>
+          <t>[ 2 ] Требуется профилактическая чистка (внутренняя/внешняя)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="inlineStr">
+        <is>
+          <t>[ 3 ] Требуется плановое ТО (замена роликов, чистка лазера)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="inlineStr">
+        <is>
+          <t>[ 4 ] Требуется замена ЗИП (указать что: _____________________)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr">
+        <is>
+          <t>[ 5 ] Требуется замена картриджа / тонера</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="inlineStr">
+        <is>
+          <t>[ 6 ] Требуется калибровка цвета (для цветных аппаратов)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr">
+        <is>
+          <t>[ 7 ] Требуется замена термоузла / печки</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="inlineStr">
+        <is>
+          <t>[ 8 ] Требуется перепрошивка / обновление встроенного ПО</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr">
+        <is>
+          <t>[ 9 ] Требуется перемещение в другую локацию / кабинет</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>[10 ] Требуется обучение пользователя / инструктаж</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr">
+        <is>
+          <t>[11 ] Требуется эскалация в вендора / авторизованный СЦ</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="inlineStr">
+        <is>
+          <t>[12 ] Требуется списание / утилизация (обоснование: ____________)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="inlineStr">
+        <is>
+          <t>[13 ] Требуется согласование с Заказчиком (ИТ / АХО)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="inlineStr">
+        <is>
+          <t>[14 ] Требуется срочная закупка расходных материалов</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="inlineStr">
+        <is>
+          <t>[15 ] Аппарат временно выведен из эксплуатации (до: ____________)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr">
+        <is>
+          <t>Приоритет выполнения:  🔴 Критичный  /  🟡 Средний  /  🟢 Плановый</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="inlineStr">
+        <is>
+          <t>Срок выполнения:       _____________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>ПОДПИСИ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="inlineStr">
+        <is>
+          <t>Антон: _______________     Александр: _______________</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="inlineStr">
+        <is>
+          <t>═══════════════════════════════════════════════════════════════</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -593,7 +1122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -602,199 +1131,511 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ЧЕК-ЛИСТ ПРОВЕРКИ ОРГТЕХНИКИ</t>
+          <t>┌─────────────────────────────────────────────────────────────┐</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Организация: Этажи</t>
+          <t>│ ЧЕК-ЛИСТ БАЗОВОЙ ПРОВЕРКИ АППАРАТА (5-7 минут)              │</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr"/>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>└─────────────────────────────────────────────────────────────┘</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Дата проверки: 22.06.2026</t>
-        </is>
-      </c>
+      <c r="A4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr"/>
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>═══════════════════════════════════════════════════════════════</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Инвентарный номер: 67+</t>
+          <t>БЛОК А. РЕКВИЗИТЫ АППАРАТА (для дальнейшего анализа)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Модель: Kyocera ECOSYS M3040dn</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Серийный номер: LS67Y43279</t>
+          <t xml:space="preserve">Модель:                  Kyocera ECOSYS M3040dn               </t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Местоположение: Риелторы (Тюмень)</t>
+          <t xml:space="preserve">Серийный номер:          LS67Y43279                           </t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Офис: Тюмень</t>
+          <t xml:space="preserve">Инвентарный номер:       67+                                  </t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Подразделение: Риелторы</t>
+          <t xml:space="preserve">Локация (офис/кабинет):  Риелторы (Тюмень)                    </t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr"/>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Модель картриджа:        _____________________________________</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Проверка:</t>
+          <t>Текущий ресурс картриджа (%): ________________________________</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>[ ] Модель соответствует учетным данным. Факт: Kyocera ECOSYS M3040dn</t>
+          <t>Дата последнего ТО:      _____________________________________</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>[ ] Серийный номер соответствует. Факт: LS67Y43279</t>
+          <t>Дата последней замены ЗИП: ___________________________________</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>[ ] Инвентарный номер соответствует. Факт: 67+</t>
+          <t>Ответственный у Заказчика: ___________________________________</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>[ ] Место размещения соответствует. Факт: Риелторы (Тюмень)</t>
+          <t>Контакт (тел/email):     _____________________________________</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>[ ] Офис соответствует. Факт: Тюмень</t>
-        </is>
-      </c>
+      <c r="A18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>[ ] Подразделение соответствует. Факт: Риелторы</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>[ ] Счетчик (предыдущий месяц) зафиксирован. Факт: 272339</t>
+          <t>БЛОК Б. ПРОВЕРКА ПО ШАГАМ</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>[ ] Счетчик (отчетный месяц) зафиксирован. Факт: 272864</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>[ ] Кол-во отпечатков проверено. Факт: 525</t>
-        </is>
-      </c>
+      <c r="A22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>[ ] Устройство включено и исправно</t>
+          <t>ШАГ 1. ВНЕШНИЙ ОСМОТР (30 сек)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>[ ] Печать / сканирование выполняется</t>
+          <t xml:space="preserve">  □ Корпус, крышки, лотки — визуально целые</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">[ ] Ответственный сотрудник определен. Факт: </t>
+          <t xml:space="preserve">  □ Кабели подключены надежно, без перегибов</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>[ ] Внешний вид и комплектность в норме</t>
+          <t xml:space="preserve">  □ Вокруг аппарата чисто, нет мусора, скрепок, скоб</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>[ ] Замечания отсутствуют</t>
-        </is>
-      </c>
+      <c r="A27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr"/>
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>ШАГ 2. СЧЕТЧИКИ (1 мин)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Проверил: __________________ / __________________</t>
+          <t xml:space="preserve">  □ Открыть меню → Отчет → Страница состояния (Kyocera)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>Подпись ответственного: __________________</t>
+          <t xml:space="preserve">     или Меню → Reports → Usage Report (HP)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr"/>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Записать: Total / ЧБ / Цвет / Сканер</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Сверить с данными в файле "Этажи покопийка AI.xlsx"</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     (расхождение &gt; 5% — пометить в карточке)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>ШАГ 3. ТЕСТОВАЯ ПЕЧАТЬ (1 мин)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Распечатать тестовую страницу из встроенного меню</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Оценить: плотность, полосы, фон, регистрация</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Проверить закрепление тонера (провести пальцем)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Для цветных — напечатать страницу качества цвета</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>ШАГ 4. ТЕСТ СКАНИРОВАНИЯ (1 мин)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Положить лист A4 на стекло / в ADF</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Отсканировать на email / в сетевую папку</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Проверить: нет полос, захват ADF без перекоса</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>ШАГ 5. ФИЗИКА (1-2 мин)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Открыть переднюю крышку, заглянуть внутрь</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Осмотреть ролики захвата (лысые? грязные?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Осмотреть термоузел (следы тонера, нагар?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Проверить дуплекс (нет ли замятой бумаги)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Понюхать (запах гари = проблема с печкой)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>ШАГ 6. СУБЪЕКТИВНАЯ ОЦЕНКА (30 сек)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Оценить физическое состояние (1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Оценить качество печати (1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Оценить качество сканирования (1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Выставить общую оценку (1-5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>ШАГ 7. ФИКСАЦИЯ В КАРТОЧКЕ</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Заполнить все поля карточки аппарата</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Отметить все применимые пункты "План действий"</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Указать приоритет и срок выполнения</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  □ Сфотографировать дефекты (если есть)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>═══════════════════════════════════════════════════════════════</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>🚨 КРАСНЫЕ ФЛАГИ (немедленная эскалация Наталье, руководителю):</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Аппарат не включается / нет реакции</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Счетчик не изменился с прошлого месяца (0 отпечатков)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Сильный запах гари, дым</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Треск, скрежет, посторонние звуки</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Явное физическое повреждение корпуса/лотков</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Оценка "1" по любому из параметров</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Аппарат отсутствует на месте (пропажа / перемещение без согласования)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Конфликт с Заказчиком / отказ в доступе</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Риск срыва SLA (критичный фронт-офис не работает)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr">
+        <is>
+          <t>Канал эскалации: мессенджер MAX → чат "Этажи_Сервис"</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="inlineStr">
+        <is>
+          <t>Время реакции Натальи: до 30 минут в рабочее время</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr">
+        <is>
+          <t>═══════════════════════════════════════════════════════════════</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -807,7 +1648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -816,24 +1657,28 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ ПО ОРГТЕХНИКЕ</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Организация: Этажи</t>
+          <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ О ХОДЕ ПЕРЕДАЧИ ДЕЛ</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr"/>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Дата: 22.06.2026  Инженер: Александр</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Дата: 22.06.2026</t>
+          <t>═══════════════════════════════════════════════════════════════</t>
         </is>
       </c>
     </row>
@@ -843,42 +1688,42 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Инвентарный номер: 67+</t>
+          <t>1. ЛОКАЦИЯ ДНЯ:</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Модель: Kyocera ECOSYS M3040dn</t>
+          <t xml:space="preserve">   Риелторы (Тюмень)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Серийный номер: LS67Y43279</t>
+          <t>2. СТАТУС ПО ОЦЕНКАМ (сводка за день):</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Местоположение: Риелторы (Тюмень)</t>
+          <t xml:space="preserve">   🟢 Оценка 4-5 (хорошее/отличное): _____ шт.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Офис: Тюмень</t>
+          <t xml:space="preserve">   🟡 Оценка 3 (удовлетворительное):   _____ шт.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Подразделение: Риелторы</t>
+          <t xml:space="preserve">   🔴 Оценка 1-2 (требует внимания):   _____ шт.</t>
         </is>
       </c>
     </row>
@@ -888,70 +1733,95 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Показания на начало периода: 272339</t>
+          <t>3. КРАСНЫЕ ФЛАГИ (эскалация Наталье):</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Показания на конец периода: 272864</t>
+          <t xml:space="preserve">   [ ] Нет</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Кол-во отпечатков за период: 525</t>
+          <t xml:space="preserve">   [ ] Да (кол-во: _____ шт.)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr"/>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Краткое описание:</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ответственный: </t>
+          <t xml:space="preserve">   ___________________________________________________________</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ___________________________________________________________</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>Состояние оборудования: Исправно / Неисправно</t>
-        </is>
-      </c>
+      <c r="A19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Комментарий:</t>
+          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr"/>
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ___________________________________________________________</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Подпись ответственного: __________________</t>
+          <t xml:space="preserve">   ___________________________________________________________</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>Подпись принявшего отчет: __________________</t>
-        </is>
-      </c>
+      <c r="A23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr"/>
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>5. ПЛАН НА ЗАВТРА:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Локация: _________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>═══════════════════════════════════════════════════════════════</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adjust xlsx layout: counters split, checkboxes in right column
- Counters: separate Значение and Ед. (стр.) columns
- Checklist items: description left, ☐ mark in Отметка column on right
- Rating rows: 1-5 scale in Отметка column

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/TEST_Sample_Device_Package.xlsx
+++ b/equipment-templates/output/TEST_Sample_Device_Package.xlsx
@@ -415,13 +415,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,6 +443,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Отметка</t>
         </is>
       </c>
@@ -459,6 +465,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -477,6 +484,7 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,6 +503,7 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -513,6 +522,7 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -527,6 +537,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -541,6 +552,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -555,6 +567,7 @@
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -573,6 +586,7 @@
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -591,6 +605,7 @@
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -609,6 +624,7 @@
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -627,6 +643,7 @@
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -641,6 +658,7 @@
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -655,6 +673,7 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -669,6 +688,7 @@
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -683,6 +703,7 @@
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -697,6 +718,7 @@
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -711,6 +733,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -725,6 +748,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -739,6 +763,7 @@
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -753,6 +778,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -767,6 +793,7 @@
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -781,6 +808,7 @@
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -795,6 +823,7 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -809,6 +838,7 @@
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -823,10 +853,15 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>272864       стр.</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>272864</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>стр.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -840,7 +875,12 @@
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>стр.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -854,7 +894,12 @@
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>стр.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -868,7 +913,12 @@
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>стр.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -883,10 +933,15 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>525          стр.</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>525</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>стр.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -901,6 +956,7 @@
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -915,6 +971,7 @@
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -929,6 +986,11 @@
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -943,6 +1005,11 @@
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -957,6 +1024,11 @@
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -971,6 +1043,11 @@
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -985,6 +1062,11 @@
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -999,6 +1081,11 @@
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1013,6 +1100,11 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1027,6 +1119,7 @@
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1041,6 +1134,7 @@
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1055,6 +1149,11 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1069,6 +1168,11 @@
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1081,8 +1185,17 @@
           <t>Нет "волн" и повторяющихся дефектов (шаг дефекта: _____ мм)</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>мм)</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1097,6 +1210,11 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1111,6 +1229,11 @@
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1125,6 +1248,7 @@
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1139,6 +1263,7 @@
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1153,6 +1278,11 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1167,6 +1297,11 @@
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1181,6 +1316,11 @@
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1195,6 +1335,11 @@
       </c>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1209,6 +1354,7 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1223,6 +1369,7 @@
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1237,6 +1384,7 @@
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1251,6 +1399,7 @@
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1265,6 +1414,7 @@
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1279,6 +1429,7 @@
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1293,6 +1444,7 @@
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1307,11 +1459,12 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Оценка</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1319,17 +1472,18 @@
           <t>Физическое состояние</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
         <is>
           <t>[ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Оценка</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1337,17 +1491,18 @@
           <t>Качество печати</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
         <is>
           <t>[ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Оценка</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1355,17 +1510,18 @@
           <t>Качество сканирования</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
         <is>
           <t>[ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Оценка</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1373,12 +1529,13 @@
           <t>Общая оценка</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
         <is>
           <t>[ 1 ] [ 2 ] [ 3 ] [ 4 ] [ 5 ]</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1393,6 +1550,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1407,6 +1565,7 @@
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1421,6 +1580,7 @@
       </c>
       <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1435,6 +1595,7 @@
       </c>
       <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1449,6 +1610,7 @@
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1463,6 +1625,7 @@
       </c>
       <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1477,6 +1640,7 @@
       </c>
       <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1491,6 +1655,7 @@
       </c>
       <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1509,6 +1674,7 @@
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1523,6 +1689,7 @@
       </c>
       <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1537,6 +1704,7 @@
       </c>
       <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1551,6 +1719,7 @@
       </c>
       <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1565,6 +1734,7 @@
       </c>
       <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1579,6 +1749,7 @@
       </c>
       <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1593,6 +1764,7 @@
       </c>
       <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1607,6 +1779,7 @@
       </c>
       <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1625,6 +1798,7 @@
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1639,6 +1813,7 @@
       </c>
       <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1653,6 +1828,7 @@
       </c>
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1671,6 +1847,7 @@
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1689,6 +1866,7 @@
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1703,6 +1881,7 @@
       </c>
       <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1717,6 +1896,7 @@
       </c>
       <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1729,8 +1909,13 @@
           <t>Антон</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Александр:</t>
+        </is>
+      </c>
       <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1745,6 +1930,7 @@
       </c>
       <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1757,13 +1943,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1784,6 +1971,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Отметка</t>
         </is>
       </c>
@@ -1801,6 +1993,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1815,6 +2008,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1829,6 +2023,7 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1843,6 +2038,7 @@
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1857,6 +2053,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1871,6 +2068,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1889,6 +2087,7 @@
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1907,6 +2106,7 @@
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1925,6 +2125,7 @@
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1943,6 +2144,7 @@
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1957,6 +2159,7 @@
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1971,6 +2174,7 @@
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1985,6 +2189,7 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1999,6 +2204,7 @@
       </c>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2013,6 +2219,7 @@
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2027,6 +2234,7 @@
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2041,6 +2249,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2055,6 +2264,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2069,6 +2279,7 @@
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2083,6 +2294,7 @@
       </c>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2097,6 +2309,11 @@
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2111,6 +2328,11 @@
       </c>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2125,6 +2347,11 @@
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2139,6 +2366,7 @@
       </c>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2153,6 +2381,11 @@
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2167,6 +2400,7 @@
       </c>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2181,6 +2415,11 @@
       </c>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2195,6 +2434,11 @@
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2209,6 +2453,7 @@
       </c>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2223,6 +2468,7 @@
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2237,6 +2483,11 @@
       </c>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2251,6 +2502,11 @@
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2265,6 +2521,11 @@
       </c>
       <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2279,6 +2540,11 @@
       </c>
       <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2293,6 +2559,7 @@
       </c>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2307,6 +2574,11 @@
       </c>
       <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2321,6 +2593,11 @@
       </c>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2335,6 +2612,11 @@
       </c>
       <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2349,6 +2631,7 @@
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2363,6 +2646,11 @@
       </c>
       <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2377,6 +2665,11 @@
       </c>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2391,6 +2684,11 @@
       </c>
       <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2405,6 +2703,11 @@
       </c>
       <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2419,6 +2722,11 @@
       </c>
       <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2433,6 +2741,7 @@
       </c>
       <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2447,6 +2756,11 @@
       </c>
       <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2461,6 +2775,11 @@
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2475,6 +2794,11 @@
       </c>
       <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2489,6 +2813,11 @@
       </c>
       <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2503,6 +2832,7 @@
       </c>
       <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2517,6 +2847,11 @@
       </c>
       <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2531,6 +2866,11 @@
       </c>
       <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2545,6 +2885,11 @@
       </c>
       <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2559,6 +2904,11 @@
       </c>
       <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2573,6 +2923,7 @@
       </c>
       <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2587,6 +2938,7 @@
       </c>
       <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2601,6 +2953,7 @@
       </c>
       <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2615,6 +2968,7 @@
       </c>
       <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2629,6 +2983,7 @@
       </c>
       <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2643,6 +2998,7 @@
       </c>
       <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2657,6 +3013,7 @@
       </c>
       <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2671,6 +3028,7 @@
       </c>
       <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2685,6 +3043,7 @@
       </c>
       <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2699,6 +3058,7 @@
       </c>
       <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2713,6 +3073,7 @@
       </c>
       <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2731,6 +3092,7 @@
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2749,6 +3111,7 @@
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2763,6 +3126,7 @@
       </c>
       <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2775,13 +3139,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2802,6 +3167,11 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Отметка</t>
         </is>
       </c>
@@ -2819,6 +3189,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2833,6 +3204,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2851,6 +3223,7 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2869,6 +3242,7 @@
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2883,6 +3257,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2897,6 +3272,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2915,6 +3291,7 @@
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2929,6 +3306,7 @@
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2943,6 +3321,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2957,6 +3336,7 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2971,6 +3351,7 @@
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2985,6 +3366,7 @@
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2999,6 +3381,11 @@
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3011,8 +3398,17 @@
           <t>Да (кол-во: _____ шт.)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>шт.)</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3027,6 +3423,7 @@
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3041,6 +3438,7 @@
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3055,6 +3453,7 @@
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3069,6 +3468,7 @@
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3083,6 +3483,7 @@
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix checkbox row value parsing for defect step line
Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/TEST_Sample_Device_Package.xlsx
+++ b/equipment-templates/output/TEST_Sample_Device_Package.xlsx
@@ -1185,11 +1185,7 @@
           <t>Нет "волн" и повторяющихся дефектов (шаг дефекта: _____ мм)</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>мм)</t>
-        </is>
-      </c>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
@@ -3398,11 +3394,7 @@
           <t>Да (кол-во: _____ шт.)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>шт.)</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>

</xml_diff>